<commit_message>
docs(spec): label static-only rows Verified (static); remove old edition dir
- split Status into Verified (108, executed Vitest/SQL-contract) and
  Verified (static) (31, static code read where no executable surface exists);
- delete the 2026-06-24 historical snapshot dir docs/behavioral-spec/ and drop
  the remaining living references to it (WORKFLOW.md, docs/spec/README.md);
- regenerate the XLSX from the CSV.

Docs-only; no code or schema change.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HfqTC4vpYxaufPZAKxTtQB
</commit_message>
<xml_diff>
--- a/docs/spec/2026-07-02-behavioral-spec.xlsx
+++ b/docs/spec/2026-07-02-behavioral-spec.xlsx
@@ -461,7 +461,7 @@
         <v>Login.tsx form calls useAuth.signIn -&gt; supabase.auth.signInWithPassword on the internal client; useAuth loads the user_profiles row and exposes profile/capabilities; a missing or inactive profile keeps the user out of protected routes; on success Login.tsx navigates to /painel itself (an already-authenticated visitor is redirected by a Navigate guard); errors shown inline.</v>
       </c>
       <c r="E2" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F2" t="str">
         <v>-</v>
@@ -557,7 +557,7 @@
         <v>src/services/supabase.ts creates two clients: supabase (staff) and supabasePortal with its own storageKey ('td-portal-auth') and detectSessionInUrl:false; the sessions coexist and logging out of one does not drop the other.</v>
       </c>
       <c r="E5" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F5" t="str">
         <v>-</v>
@@ -621,7 +621,7 @@
         <v>RLS (010_rls_by_role.sql + later fixes): self/admin SELECT; a user updates only their own row and only while active; INSERT/DELETE admin-only. Helpers is_active_user()/is_admin()/current_user_role() underpin all role-based policies.</v>
       </c>
       <c r="E7" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F7" t="str">
         <v>-</v>
@@ -653,7 +653,7 @@
         <v>prevent_user_profile_privilege_escalation() BEFORE UPDATE on user_profiles rejects a user changing their own role or active flag; service_role remains allowed for provisioning.</v>
       </c>
       <c r="E8" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F8" t="str">
         <v>-</v>
@@ -877,7 +877,7 @@
         <v>The catch-all route in src/App.tsx renders Navigate to /painel with replace; the destination then applies the normal auth guards.</v>
       </c>
       <c r="E15" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F15" t="str">
         <v>-</v>
@@ -909,7 +909,7 @@
         <v>count_distinct_containers() -&gt; bigint (045_count_distinct_containers_fn.sql), STABLE SECURITY INVOKER, PUBLIC revoked, authenticated granted; read-only aggregate. No frontend caller exists in src today.</v>
       </c>
       <c r="E16" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F16" t="str">
         <v>-</v>
@@ -941,7 +941,7 @@
         <v>010_rls_by_role.sql: active users read/insert/update alerts; only admin deletes; alert writers include overdue detection and portal dispute flows.</v>
       </c>
       <c r="E17" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F17" t="str">
         <v>-</v>
@@ -973,7 +973,7 @@
         <v>014_lock_down_financial_reads_and_audit_writes.sql: active users read; INSERT requires active profile and changed_by=auth.uid(); UPDATE/DELETE admin-only. audit_logs feeds B/L timeline, voyage timeline and admin observability.</v>
       </c>
       <c r="E18" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F18" t="str">
         <v>-</v>
@@ -1005,7 +1005,7 @@
         <v>pg_cron job cleanup-portal-sessions (03:00 UTC, 041_rls_missing_tables.sql) deletes legacy portal sessions expired for more than one day.</v>
       </c>
       <c r="E19" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F19" t="str">
         <v>-</v>
@@ -1037,7 +1037,7 @@
         <v>pg_cron job cleanup-provision-rate-limit (03:30 UTC, 053_security_hardening.sql) removes provision-portal-user rate-limit rows older than 2 days.</v>
       </c>
       <c r="E20" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F20" t="str">
         <v>-</v>
@@ -1325,7 +1325,7 @@
         <v>trg_voyage_schedule_snapshot AFTER INSERT on audit_logs (POD/POL events) updates voyages JSONB snapshot; 052 fixed JSON null handling so a null new_value does not violate NOT NULL.</v>
       </c>
       <c r="E29" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F29" t="str">
         <v>-</v>
@@ -1485,7 +1485,7 @@
         <v>124_vessel_schedules.sql (+ 139 grants): SELECT for any authenticated (portal-compatible by design); INSERT/UPDATE require active internal user; DELETE admin. ended_vessels: SELECT authenticated; INSERT active; DELETE admin; no UPDATE policy exists.</v>
       </c>
       <c r="E34" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F34" t="str">
         <v>-</v>
@@ -1837,7 +1837,7 @@
         <v>validate_bl_breakbulk_item_parent() BEFORE INSERT/UPDATE on bl_breakbulk_items (006_breakbulk_module.sql) rejects items whose parent B/L cargo mode is not carga_solta.</v>
       </c>
       <c r="E45" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F45" t="str">
         <v>-</v>
@@ -1933,7 +1933,7 @@
         <v>validate_vehicle_relationships() BEFORE INSERT/UPDATE on vehicles (004_vehicles.sql; search_path fixed later) normalizes fields and rejects incoherent voyage/B/L/container combinations.</v>
       </c>
       <c r="E48" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F48" t="str">
         <v>-</v>
@@ -2189,7 +2189,7 @@
         <v>Final state of 010: bls, bl_containers, bl_breakbulk_items — active users read/insert/update; admin deletes. bls carries review gate, promotion and billing guards via triggers; bl_containers delete additionally blocked by service-level dependency checks.</v>
       </c>
       <c r="E56" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F56" t="str">
         <v>-</v>
@@ -2477,7 +2477,7 @@
         <v>mark_bl_charges_reviewed(text,uuid) -&gt; jsonb (019; DEFINER; active user): moves calculations/B/L to reviewed and audits; hooks invalidate lines, B/Ls and pendencies.</v>
       </c>
       <c r="E65" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F65" t="str">
         <v>-</v>
@@ -2541,7 +2541,7 @@
         <v>mark_bl_ready_and_create_invoice(text,bigint,date,text,uuid) -&gt; jsonb (102_mark_ready_and_invoice_atomic.sql; INVOKER; active+admin): marks ready and creates invoice+ledger in one transaction; any failure rolls back both.</v>
       </c>
       <c r="E67" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F67" t="str">
         <v>-</v>
@@ -2701,7 +2701,7 @@
         <v>guard_container_bl_without_containers() AFTER I/U on bls (064) creates a synthetic pendency so an empty container B/L cannot stay calculated/ready; ensure_container_bl_charge_status_default() (065) converts NULL charge_status of CNTR B/Ls to not_calculated; populate_charge_calculation_billing_metadata() (025) fills manifest and commercial-rule version on charge_calculations.</v>
       </c>
       <c r="E72" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F72" t="str">
         <v>-</v>
@@ -2733,7 +2733,7 @@
         <v>charge_tables, charge_table_items, customer_rate_overrides: all operations admin-only (010+014). charge_calculations: SELECT admin (014), INSERT/UPDATE active (010), DELETE admin. customer_reconciliation_queue guarded via RPCs.</v>
       </c>
       <c r="E73" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F73" t="str">
         <v>-</v>
@@ -3149,7 +3149,7 @@
         <v>assign_invoice_number() BEFORE INSERT on invoices (003) fills the annual sequential number; fn_block_invoice_overdue_customer() (031) blocks a new invoice when the customer has an overdue local invoice; prevent_duplicate_active_invoice_bl_link() (064) rejects a second active/paid link for the same B/L.</v>
       </c>
       <c r="E86" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F86" t="str">
         <v>-</v>
@@ -3181,7 +3181,7 @@
         <v>pg_cron job mark-overdue-invoices (06:00 UTC; 031) runs mark_overdue_invoices() over local invoices; demurrage was removed from overdue enforcement by 157_demurrage_drop_overdue.sql (demurrage has no due_date/overdue).</v>
       </c>
       <c r="E87" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F87" t="str">
         <v>-</v>
@@ -3341,7 +3341,7 @@
         <v>invoices, payments, invoice_bls, billing_batches (SELECT active per 041), bl_receivables and invoice_receivable_links: financial families are admin-only for writes (and mostly for reads) per 010+014+020 and the ledger migrations; operational surfaces read through RPCs.</v>
       </c>
       <c r="E92" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F92" t="str">
         <v>-</v>
@@ -3437,7 +3437,7 @@
         <v>src/App.tsx renders Navigate to /demurrage with replace.</v>
       </c>
       <c r="E95" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F95" t="str">
         <v>-</v>
@@ -3661,7 +3661,7 @@
         <v>Edge Function recalc-demurrage-ptax: requires Authorization bearer exactly equal to SUPABASE_SERVICE_ROLE_KEY (timing-safe compare); queries BCB CotacaoDolarPeriodo for the last ~10 days, top 1 by dataHoraCotacao desc (never 'today only', so weekends/holidays return the latest quote); passes raw cotacaoVenda to recalculate_demurrage_invoices (markup applied in DB); aborts with error only on HTTP/network failure or empty period; designed to be scheduled weekdays ~14h BRT.</v>
       </c>
       <c r="E102" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F102" t="str">
         <v>-</v>
@@ -3853,7 +3853,7 @@
         <v>reconcile_invoice_payment_by_txid(text,numeric,timestamptz) -&gt; jsonb (067; DEFINER; active+admin): strict TXID match; records payment/settlement and updates invoice/receivables.</v>
       </c>
       <c r="E108" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F108" t="str">
         <v>-</v>
@@ -3949,7 +3949,7 @@
         <v>src/App.tsx renders Navigate to /reconciliacao with replace.</v>
       </c>
       <c r="E111" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F111" t="str">
         <v>-</v>
@@ -4365,7 +4365,7 @@
         <v>trg_notify_invoice_issued (invoices status -&gt; issued), trg_notify_demurrage_issued (demurrage_invoices) and trg_notify_dispute_responded (dispute_status -&gt; resolvido) insert portal_notifications rows (116_portal_fase2_notifications_disputes_profile.sql); this in-app path is the active customer notification mechanism (email is off by decision).</v>
       </c>
       <c r="E124" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F124" t="str">
         <v>-</v>
@@ -4429,7 +4429,7 @@
         <v>notify-invoice-issued: bearer must equal SUPABASE_SERVICE_ROLE_KEY (timing-safe); accepts absent Origin or Origin == SUPABASE_URL; service role re-reads invoices/customers/customer_contacts (no DB writes) and sends via Resend; missing recipient/key -&gt; skipped/sent:false; auth failure 401; Resend/parse failure 500. No functions.invoke caller exists in src and no webhook is configured in the repo — inactive by decision; customer notification is in-app via trg_notify_invoice_issued.</v>
       </c>
       <c r="E126" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F126" t="str">
         <v>-</v>
@@ -4621,7 +4621,7 @@
         <v>prevent_duplicate_active_invoice_granite_bl_link() BEFORE I/U on invoice_granite_bls (064) rejects a second active/paid link for the same granite B/L.</v>
       </c>
       <c r="E132" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F132" t="str">
         <v>-</v>
@@ -4653,7 +4653,7 @@
         <v>granite_manifests, granite_bls, granite_bl_charges, granite_rates (042 final + 050 alignment): active users read/insert/update; admin deletes; invoice_granite_bls follows the financial family.</v>
       </c>
       <c r="E133" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F133" t="str">
         <v>-</v>
@@ -4877,7 +4877,7 @@
         <v>customers and customer_contacts (010 final): active users read/insert/update; admin deletes; Portal profile writes go only through portal_update_profile; contact email participates in the review gate.</v>
       </c>
       <c r="E140" t="str">
-        <v>Verified</v>
+        <v>Verified (static)</v>
       </c>
       <c r="F140" t="str">
         <v>-</v>
@@ -4905,7 +4905,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <cols>
     <col min="1" max="1" width="36.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -4945,15 +4945,23 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>Status: Verified (static)</v>
+      </c>
+      <c r="B5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
         <v>Status: Verified</v>
       </c>
-      <c r="B5">
-        <v>139</v>
+      <c r="B6">
+        <v>108</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: omissao de escala, transbordo e COD
</commit_message>
<xml_diff>
--- a/docs/spec/2026-07-02-behavioral-spec.xlsx
+++ b/docs/spec/2026-07-02-behavioral-spec.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Behavioral Spec'!$A$1:$J$140</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Behavioral Spec'!$A$1:$J$143</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J140"/>
+  <dimension ref="A1:J143"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -1113,7 +1113,7 @@
         <v>Vitest: Viagens.behavior.test.tsx; VoyageSectionCards.test.tsx; voyageTimeline.behavior.test.ts</v>
       </c>
       <c r="I22" t="str">
-        <v>src/pages/Viagens.tsx; src/pages/viagensHelpers.ts; src/services/voyageTimeline.ts</v>
+        <v>src/pages/Viagens.tsx; src/services/voyageSummaries.ts; src/services/voyageTimeline.ts</v>
       </c>
       <c r="J22" t="str">
         <v>-</v>
@@ -4895,10 +4895,106 @@
         <v>Verified by code read — SQL/trigger/cron/edge or live-DB RLS surface with no executable assertion in this environment (static is the strongest method available).</v>
       </c>
     </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>VOY-OMIT-01</v>
+      </c>
+      <c r="B141" t="str">
+        <v>Viagens</v>
+      </c>
+      <c r="C141" t="str">
+        <v>As an operator I omit a port call and keep traceability</v>
+      </c>
+      <c r="D141" t="str">
+        <v>OmitEscalaModal calls omit_voyage_escala; the RPC writes voyage_omissions, audit_logs field omitted=true, default bl_transshipments rows and a transshipment portal notification; omitted PODs are ignored by next-call and completion derivations.</v>
+      </c>
+      <c r="E141" t="str">
+        <v>Verified</v>
+      </c>
+      <c r="F141" t="str">
+        <v>-</v>
+      </c>
+      <c r="G141" t="str">
+        <v>-</v>
+      </c>
+      <c r="H141" t="str">
+        <v>Vitest: voyageOmissionsMigration.test.ts; voyageSummaries.omitted.test.ts; voyageRouteSchedules.omitted.test.ts</v>
+      </c>
+      <c r="I141" t="str">
+        <v>src/components/voyages/OmitEscalaModal.tsx; src/services/transshipments.ts; src/services/voyageSummaries.ts; src/services/voyageRouteSchedules.ts; supabase/migrations/174_voyage_omissions_transshipments.sql</v>
+      </c>
+      <c r="J141" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>VOY-OMIT-02</v>
+      </c>
+      <c r="B142" t="str">
+        <v>Portal</v>
+      </c>
+      <c r="C142" t="str">
+        <v>As a portal customer I do not see omitted PODs in the public schedule</v>
+      </c>
+      <c r="D142" t="str">
+        <v>portal_ship_schedule includes omitted_pods and filters audit_logs field_name='omitted' alongside deleted pods before returning the schedule projection.</v>
+      </c>
+      <c r="E142" t="str">
+        <v>Verified</v>
+      </c>
+      <c r="F142" t="str">
+        <v>-</v>
+      </c>
+      <c r="G142" t="str">
+        <v>-</v>
+      </c>
+      <c r="H142" t="str">
+        <v>Vitest: portalShipScheduleOmitted.test.ts</v>
+      </c>
+      <c r="I142" t="str">
+        <v>supabase/migrations/175_portal_ship_schedule_hide_omitted.sql; src/services/portalScheduleVoyages.ts</v>
+      </c>
+      <c r="J142" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>VOY-COD-01</v>
+      </c>
+      <c r="B143" t="str">
+        <v>Viagens</v>
+      </c>
+      <c r="C143" t="str">
+        <v>As an operator I choose transshipment or COD per B/L</v>
+      </c>
+      <c r="D143" t="str">
+        <v>TransshipmentPanel calls set_bl_transshipment or set_bl_cod; transshipment stores third-party vessel reference, while COD clears those fields and updates bls.pod to the discharge port through audited RPCs.</v>
+      </c>
+      <c r="E143" t="str">
+        <v>Verified</v>
+      </c>
+      <c r="F143" t="str">
+        <v>-</v>
+      </c>
+      <c r="G143" t="str">
+        <v>-</v>
+      </c>
+      <c r="H143" t="str">
+        <v>Vitest: transshipments.test.ts</v>
+      </c>
+      <c r="I143" t="str">
+        <v>src/components/voyages/TransshipmentPanel.tsx; src/hooks/useTransshipments.ts; src/services/transshipments.ts; supabase/migrations/174_voyage_omissions_transshipments.sql</v>
+      </c>
+      <c r="J143" t="str">
+        <v>-</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J140"/>
+  <autoFilter ref="A1:J143"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J140"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J143"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4924,7 +5020,7 @@
         <v>Source CSV</v>
       </c>
       <c r="B2" t="str">
-        <v>docs/spec/2026-07-02-behavioral-spec.csv</v>
+        <v>C:\Users\Lucca\Downloads\transhipping-desk2\docs\spec\2026-07-02-behavioral-spec.csv</v>
       </c>
     </row>
     <row r="3">
@@ -4932,7 +5028,7 @@
         <v>Generated</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-07-02</v>
+        <v>2026-07-09</v>
       </c>
     </row>
     <row r="4">
@@ -4940,7 +5036,7 @@
         <v>Total stories</v>
       </c>
       <c r="B4">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5">
@@ -4956,7 +5052,7 @@
         <v>Status: Verified</v>
       </c>
       <c r="B6">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>